<commit_message>
Add smoking & ulcer as covariates
</commit_message>
<xml_diff>
--- a/results/pooled_results_OR_multi_exposure_models.xlsx
+++ b/results/pooled_results_OR_multi_exposure_models.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Keiji\Documents\Research\ahs_fibromyalgia\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1DD6887-C5C3-4CE3-8780-63608A6C8AD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EAED8F59-528F-4B6F-8591-D890FBF363DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{797B858C-DA94-466A-A931-46BE830858D9}"/>
   </bookViews>
@@ -323,6 +323,9 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="2" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -330,9 +333,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="2" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -711,30 +711,30 @@
       <c r="C4" s="5"/>
     </row>
     <row r="5" spans="2:22" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D5" s="18" t="s">
+      <c r="D5" s="19" t="s">
         <v>32</v>
       </c>
-      <c r="E5" s="19"/>
-      <c r="F5" s="19"/>
-      <c r="G5" s="20"/>
-      <c r="I5" s="18" t="s">
+      <c r="E5" s="20"/>
+      <c r="F5" s="20"/>
+      <c r="G5" s="21"/>
+      <c r="I5" s="19" t="s">
         <v>33</v>
       </c>
-      <c r="J5" s="19"/>
-      <c r="K5" s="19"/>
-      <c r="L5" s="20"/>
-      <c r="N5" s="18" t="s">
+      <c r="J5" s="20"/>
+      <c r="K5" s="20"/>
+      <c r="L5" s="21"/>
+      <c r="N5" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="O5" s="19"/>
-      <c r="P5" s="19"/>
-      <c r="Q5" s="20"/>
-      <c r="S5" s="18" t="s">
+      <c r="O5" s="20"/>
+      <c r="P5" s="20"/>
+      <c r="Q5" s="21"/>
+      <c r="S5" s="19" t="s">
         <v>35</v>
       </c>
-      <c r="T5" s="19"/>
-      <c r="U5" s="19"/>
-      <c r="V5" s="20"/>
+      <c r="T5" s="20"/>
+      <c r="U5" s="20"/>
+      <c r="V5" s="21"/>
     </row>
     <row r="6" spans="2:22" x14ac:dyDescent="0.3">
       <c r="D6" s="9"/>
@@ -809,31 +809,31 @@
       <c r="D8" s="1">
         <v>1</v>
       </c>
-      <c r="E8" s="21" t="s">
-        <v>28</v>
-      </c>
-      <c r="F8" s="21"/>
+      <c r="E8" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="F8" s="18"/>
       <c r="I8" s="1">
         <v>1</v>
       </c>
-      <c r="J8" s="21" t="s">
-        <v>28</v>
-      </c>
-      <c r="K8" s="21"/>
+      <c r="J8" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="K8" s="18"/>
       <c r="N8" s="1">
         <v>1</v>
       </c>
-      <c r="O8" s="21" t="s">
-        <v>28</v>
-      </c>
-      <c r="P8" s="21"/>
+      <c r="O8" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="P8" s="18"/>
       <c r="S8" s="1">
         <v>1</v>
       </c>
-      <c r="T8" s="21" t="s">
-        <v>28</v>
-      </c>
-      <c r="U8" s="21"/>
+      <c r="T8" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="U8" s="18"/>
     </row>
     <row r="9" spans="2:22" x14ac:dyDescent="0.3">
       <c r="C9" s="3" t="s">
@@ -1786,15 +1786,6 @@
     <row r="45" spans="2:22" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <mergeCells count="24">
-    <mergeCell ref="T35:U35"/>
-    <mergeCell ref="O39:P39"/>
-    <mergeCell ref="E8:F8"/>
-    <mergeCell ref="J8:K8"/>
-    <mergeCell ref="O8:P8"/>
-    <mergeCell ref="T8:U8"/>
-    <mergeCell ref="E12:F12"/>
-    <mergeCell ref="J17:K17"/>
-    <mergeCell ref="T39:U39"/>
     <mergeCell ref="J42:K42"/>
     <mergeCell ref="O42:P42"/>
     <mergeCell ref="T42:U42"/>
@@ -1810,6 +1801,15 @@
     <mergeCell ref="J35:K35"/>
     <mergeCell ref="J39:K39"/>
     <mergeCell ref="O35:P35"/>
+    <mergeCell ref="T35:U35"/>
+    <mergeCell ref="O39:P39"/>
+    <mergeCell ref="E8:F8"/>
+    <mergeCell ref="J8:K8"/>
+    <mergeCell ref="O8:P8"/>
+    <mergeCell ref="T8:U8"/>
+    <mergeCell ref="E12:F12"/>
+    <mergeCell ref="J17:K17"/>
+    <mergeCell ref="T39:U39"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>